<commit_message>
Updated Excel - 13 September 2026
</commit_message>
<xml_diff>
--- a/12603165.xlsx
+++ b/12603165.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ujjwa\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C909515E-0322-4AFB-8E3D-E6D0D2C43DBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3739E068-5F37-4C5D-828C-AEE131EEE20B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -293,6 +293,15 @@
   </si>
   <si>
     <t>Had Our School Fresher's Party.</t>
+  </si>
+  <si>
+    <t>was a very heartwarming experience from the rain in the evening.</t>
+  </si>
+  <si>
+    <t>Saturday was ereally nice.</t>
+  </si>
+  <si>
+    <t>Visited DSR , and Played Football in the rain.</t>
   </si>
 </sst>
 </file>
@@ -2153,71 +2162,143 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="8"/>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
-      <c r="I30" s="10" t="str">
+    <row r="30" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A30" s="8">
+        <v>46276</v>
+      </c>
+      <c r="B30" s="9">
+        <v>190</v>
+      </c>
+      <c r="C30" s="9">
+        <v>40</v>
+      </c>
+      <c r="D30" s="9">
+        <v>80</v>
+      </c>
+      <c r="E30" s="9">
+        <v>60</v>
+      </c>
+      <c r="F30" s="9">
+        <v>200</v>
+      </c>
+      <c r="G30" s="9">
+        <v>4</v>
+      </c>
+      <c r="H30" s="9">
+        <v>650</v>
+      </c>
+      <c r="I30" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="10" t="str">
+        <v>1220</v>
+      </c>
+      <c r="J30" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="11"/>
-      <c r="L30" s="11"/>
-      <c r="M30" s="11"/>
-      <c r="N30" s="12"/>
+        <v>220</v>
+      </c>
+      <c r="K30" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="L30" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M30" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N30" s="12" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="8"/>
-      <c r="B31" s="9"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="9"/>
-      <c r="H31" s="9"/>
-      <c r="I31" s="10" t="str">
+      <c r="A31" s="8">
+        <v>46277</v>
+      </c>
+      <c r="B31" s="9">
+        <v>250</v>
+      </c>
+      <c r="C31" s="9">
+        <v>45</v>
+      </c>
+      <c r="D31" s="9">
+        <v>140</v>
+      </c>
+      <c r="E31" s="9">
+        <v>50</v>
+      </c>
+      <c r="F31" s="9">
+        <v>0</v>
+      </c>
+      <c r="G31" s="9">
+        <v>0</v>
+      </c>
+      <c r="H31" s="9">
+        <v>900</v>
+      </c>
+      <c r="I31" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="10" t="str">
+        <v>1385</v>
+      </c>
+      <c r="J31" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="11"/>
-      <c r="L31" s="11"/>
-      <c r="M31" s="11"/>
-      <c r="N31" s="12"/>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="8"/>
-      <c r="B32" s="9"/>
-      <c r="C32" s="9"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="9"/>
-      <c r="G32" s="9"/>
-      <c r="H32" s="9"/>
-      <c r="I32" s="10" t="str">
+        <v>55</v>
+      </c>
+      <c r="K31" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L31" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M31" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N31" s="12" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A32" s="8">
+        <v>46278</v>
+      </c>
+      <c r="B32" s="9">
+        <v>300</v>
+      </c>
+      <c r="C32" s="9">
+        <v>10</v>
+      </c>
+      <c r="D32" s="9">
+        <v>150</v>
+      </c>
+      <c r="E32" s="9">
+        <v>130</v>
+      </c>
+      <c r="F32" s="9">
+        <v>0</v>
+      </c>
+      <c r="G32" s="9">
+        <v>0</v>
+      </c>
+      <c r="H32" s="9">
+        <v>780</v>
+      </c>
+      <c r="I32" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J32" s="10" t="str">
+        <v>1370</v>
+      </c>
+      <c r="J32" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K32" s="11"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
-      <c r="N32" s="12"/>
+        <v>70</v>
+      </c>
+      <c r="K32" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="L32" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="M32" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N32" s="12" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="8"/>

</xml_diff>

<commit_message>
Updated Excel - 14 September 2026
</commit_message>
<xml_diff>
--- a/12603165.xlsx
+++ b/12603165.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ujjwa\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\12603165-CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3739E068-5F37-4C5D-828C-AEE131EEE20B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06876F5F-E3AB-4E08-A155-1471E529DD0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="91">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -302,6 +302,9 @@
   </si>
   <si>
     <t>Visited DSR , and Played Football in the rain.</t>
+  </si>
+  <si>
+    <t>day was cool and had an average experience.</t>
   </si>
 </sst>
 </file>
@@ -2300,27 +2303,51 @@
         <v>89</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="8"/>
-      <c r="B33" s="9"/>
-      <c r="C33" s="9"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="9"/>
-      <c r="G33" s="9"/>
-      <c r="H33" s="9"/>
-      <c r="I33" s="10" t="str">
+    <row r="33" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="8">
+        <v>46279</v>
+      </c>
+      <c r="B33" s="9">
+        <v>415</v>
+      </c>
+      <c r="C33" s="9">
+        <v>45</v>
+      </c>
+      <c r="D33" s="9">
+        <v>70</v>
+      </c>
+      <c r="E33" s="9">
+        <v>40</v>
+      </c>
+      <c r="F33" s="9">
+        <v>350</v>
+      </c>
+      <c r="G33" s="9">
+        <v>7</v>
+      </c>
+      <c r="H33" s="9">
+        <v>250</v>
+      </c>
+      <c r="I33" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J33" s="10" t="str">
+        <v>1170</v>
+      </c>
+      <c r="J33" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K33" s="11"/>
-      <c r="L33" s="11"/>
-      <c r="M33" s="11"/>
-      <c r="N33" s="12"/>
+        <v>270</v>
+      </c>
+      <c r="K33" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="L33" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M33" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N33" s="12" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="8"/>

</xml_diff>

<commit_message>
Updated Excel - 18 September 2026
</commit_message>
<xml_diff>
--- a/12603165.xlsx
+++ b/12603165.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\12603165-CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06876F5F-E3AB-4E08-A155-1471E529DD0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE71341C-454C-4FC0-ABCD-661D6E0C9414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="95">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -305,6 +305,18 @@
   </si>
   <si>
     <t>day was cool and had an average experience.</t>
+  </si>
+  <si>
+    <t>I really enjoyed te day because of the less classes.</t>
+  </si>
+  <si>
+    <t>too much classes and test also.</t>
+  </si>
+  <si>
+    <t>Had a great time in playing volleyball with friends.</t>
+  </si>
+  <si>
+    <t>Day was hectic as of the 6 classes and had, my mentor meeting , I which I got some suggestions for time management.</t>
   </si>
 </sst>
 </file>
@@ -2349,93 +2361,189 @@
         <v>90</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="8"/>
-      <c r="B34" s="9"/>
-      <c r="C34" s="9"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="9"/>
-      <c r="H34" s="9"/>
-      <c r="I34" s="10" t="str">
+    <row r="34" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="8">
+        <v>46280</v>
+      </c>
+      <c r="B34" s="9">
+        <v>300</v>
+      </c>
+      <c r="C34" s="9">
+        <v>40</v>
+      </c>
+      <c r="D34" s="9">
+        <v>200</v>
+      </c>
+      <c r="E34" s="9">
+        <v>50</v>
+      </c>
+      <c r="F34" s="9">
+        <v>150</v>
+      </c>
+      <c r="G34" s="9">
+        <v>3</v>
+      </c>
+      <c r="H34" s="9">
+        <v>300</v>
+      </c>
+      <c r="I34" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J34" s="10" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J34" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K34" s="11"/>
-      <c r="L34" s="11"/>
-      <c r="M34" s="11"/>
-      <c r="N34" s="12"/>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A35" s="8"/>
-      <c r="B35" s="9"/>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="9"/>
-      <c r="H35" s="9"/>
-      <c r="I35" s="10" t="str">
+        <v>400</v>
+      </c>
+      <c r="K34" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="L34" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="M34" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N34" s="12" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35" s="8">
+        <v>46281</v>
+      </c>
+      <c r="B35" s="9">
+        <v>310</v>
+      </c>
+      <c r="C35" s="9">
+        <v>45</v>
+      </c>
+      <c r="D35" s="9">
+        <v>163</v>
+      </c>
+      <c r="E35" s="9">
+        <v>64</v>
+      </c>
+      <c r="F35" s="9">
+        <v>350</v>
+      </c>
+      <c r="G35" s="9">
+        <v>7</v>
+      </c>
+      <c r="H35" s="9">
+        <v>420</v>
+      </c>
+      <c r="I35" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J35" s="10" t="str">
+        <v>1352</v>
+      </c>
+      <c r="J35" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K35" s="11"/>
-      <c r="L35" s="11"/>
-      <c r="M35" s="11"/>
-      <c r="N35" s="12"/>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A36" s="8"/>
-      <c r="B36" s="9"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="9"/>
-      <c r="H36" s="9"/>
-      <c r="I36" s="10" t="str">
+        <v>88</v>
+      </c>
+      <c r="K35" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="L35" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="M35" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="N35" s="12" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" s="8">
+        <v>46282</v>
+      </c>
+      <c r="B36" s="9">
+        <v>250</v>
+      </c>
+      <c r="C36" s="9">
+        <v>20</v>
+      </c>
+      <c r="D36" s="9">
+        <v>284</v>
+      </c>
+      <c r="E36" s="9">
+        <v>80</v>
+      </c>
+      <c r="F36" s="9">
+        <v>200</v>
+      </c>
+      <c r="G36" s="9">
+        <v>4</v>
+      </c>
+      <c r="H36" s="9">
+        <v>180</v>
+      </c>
+      <c r="I36" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J36" s="10" t="str">
+        <v>1014</v>
+      </c>
+      <c r="J36" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K36" s="11"/>
-      <c r="L36" s="11"/>
-      <c r="M36" s="11"/>
-      <c r="N36" s="12"/>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" s="8"/>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="9"/>
-      <c r="H37" s="9"/>
-      <c r="I37" s="10" t="str">
+        <v>426</v>
+      </c>
+      <c r="K36" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L36" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M36" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N36" s="12" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+      <c r="A37" s="8">
+        <v>46283</v>
+      </c>
+      <c r="B37" s="9">
+        <v>420</v>
+      </c>
+      <c r="C37" s="9">
+        <v>45</v>
+      </c>
+      <c r="D37" s="9">
+        <v>190</v>
+      </c>
+      <c r="E37" s="9">
+        <v>120</v>
+      </c>
+      <c r="F37" s="9">
+        <v>300</v>
+      </c>
+      <c r="G37" s="9">
+        <v>6</v>
+      </c>
+      <c r="H37" s="9">
+        <v>360</v>
+      </c>
+      <c r="I37" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="10" t="str">
+        <v>1435</v>
+      </c>
+      <c r="J37" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="11"/>
-      <c r="L37" s="11"/>
-      <c r="M37" s="11"/>
-      <c r="N37" s="12"/>
+        <v>5</v>
+      </c>
+      <c r="K37" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="L37" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="M37" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N37" s="12" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="8"/>

</xml_diff>

<commit_message>
UPDATED EXCEL - 20 SEPTEMBER 2026
</commit_message>
<xml_diff>
--- a/12603165.xlsx
+++ b/12603165.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\12603165-CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE71341C-454C-4FC0-ABCD-661D6E0C9414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C386815-82E7-4B5B-B59B-443628B12D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="97">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -317,6 +317,12 @@
   </si>
   <si>
     <t>Day was hectic as of the 6 classes and had, my mentor meeting , I which I got some suggestions for time management.</t>
+  </si>
+  <si>
+    <t>Researched about some techniques of making my github profile Look innovative and good.</t>
+  </si>
+  <si>
+    <t>Tried some interesting ideas to work on for upcoming hackathon.</t>
   </si>
 </sst>
 </file>
@@ -2545,49 +2551,97 @@
         <v>94</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="8"/>
-      <c r="B38" s="9"/>
-      <c r="C38" s="9"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
-      <c r="G38" s="9"/>
-      <c r="H38" s="9"/>
-      <c r="I38" s="10" t="str">
+    <row r="38" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A38" s="8">
+        <v>46284</v>
+      </c>
+      <c r="B38" s="9">
+        <v>280</v>
+      </c>
+      <c r="C38" s="9">
+        <v>45</v>
+      </c>
+      <c r="D38" s="9">
+        <v>360</v>
+      </c>
+      <c r="E38" s="9">
+        <v>190</v>
+      </c>
+      <c r="F38" s="9">
+        <v>0</v>
+      </c>
+      <c r="G38" s="9">
+        <v>0</v>
+      </c>
+      <c r="H38" s="9">
+        <v>510</v>
+      </c>
+      <c r="I38" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="10" t="str">
+        <v>1385</v>
+      </c>
+      <c r="J38" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K38" s="11"/>
-      <c r="L38" s="11"/>
-      <c r="M38" s="11"/>
-      <c r="N38" s="12"/>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A39" s="8"/>
-      <c r="B39" s="9"/>
-      <c r="C39" s="9"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="9"/>
-      <c r="G39" s="9"/>
-      <c r="H39" s="9"/>
-      <c r="I39" s="10" t="str">
+        <v>55</v>
+      </c>
+      <c r="K38" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="L38" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="M38" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="N38" s="12" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A39" s="8">
+        <v>46285</v>
+      </c>
+      <c r="B39" s="9">
+        <v>360</v>
+      </c>
+      <c r="C39" s="9">
+        <v>45</v>
+      </c>
+      <c r="D39" s="9">
+        <v>400</v>
+      </c>
+      <c r="E39" s="9">
+        <v>180</v>
+      </c>
+      <c r="F39" s="9">
+        <v>0</v>
+      </c>
+      <c r="G39" s="9">
+        <v>0</v>
+      </c>
+      <c r="H39" s="9">
+        <v>420</v>
+      </c>
+      <c r="I39" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="10" t="str">
+        <v>1405</v>
+      </c>
+      <c r="J39" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K39" s="11"/>
-      <c r="L39" s="11"/>
-      <c r="M39" s="11"/>
-      <c r="N39" s="12"/>
+        <v>35</v>
+      </c>
+      <c r="K39" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="L39" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="M39" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="N39" s="12" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="8"/>

</xml_diff>

<commit_message>
Updated Excel - 23 September 2026
</commit_message>
<xml_diff>
--- a/12603165.xlsx
+++ b/12603165.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\12603165-CAP776\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MINOR PROJECT #1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE5FD04-F932-4F21-B082-D82B092D1E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B5F68E7-742C-4A61-8069-D78C223CA043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="100">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -187,9 +187,6 @@
     <t>5. GOOD PRACTICE</t>
   </si>
   <si>
-    <t>Ujjwal Pratap Singh</t>
-  </si>
-  <si>
     <t>MCA D1P2632</t>
   </si>
   <si>
@@ -329,6 +326,12 @@
   </si>
   <si>
     <t>Cleaned up my desktop folders and reorganized project files properly.</t>
+  </si>
+  <si>
+    <t>Ujjwal Pratap Singh</t>
+  </si>
+  <si>
+    <t>The day was Too tiring But enjoyed the Lectures.</t>
   </si>
 </sst>
 </file>
@@ -994,7 +997,7 @@
         <v>30</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>51</v>
+        <v>98</v>
       </c>
       <c r="C2" s="15"/>
       <c r="D2" s="15"/>
@@ -1011,7 +1014,7 @@
         <v>32</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C3" s="15"/>
       <c r="D3" s="15"/>
@@ -1019,7 +1022,7 @@
         <v>33</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G3" s="15"/>
     </row>
@@ -1119,16 +1122,16 @@
         <v>140</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L6" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N6" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -1165,16 +1168,16 @@
         <v>10</v>
       </c>
       <c r="K7" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L7" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M7" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N7" s="12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -1211,16 +1214,16 @@
         <v>380</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L8" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N8" s="12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -1257,16 +1260,16 @@
         <v>270</v>
       </c>
       <c r="K9" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L9" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M9" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N9" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -1303,16 +1306,16 @@
         <v>140</v>
       </c>
       <c r="K10" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L10" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M10" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N10" s="12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -1349,16 +1352,16 @@
         <v>430</v>
       </c>
       <c r="K11" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L11" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="M11" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="N11" s="12" t="s">
         <v>65</v>
-      </c>
-      <c r="M11" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="N11" s="12" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -1395,16 +1398,16 @@
         <v>260</v>
       </c>
       <c r="K12" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L12" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M12" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N12" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -1441,16 +1444,16 @@
         <v>240</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L13" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M13" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N13" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -1487,16 +1490,16 @@
         <v>480</v>
       </c>
       <c r="K14" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L14" s="11" t="s">
         <v>61</v>
-      </c>
-      <c r="L14" s="11" t="s">
-        <v>62</v>
       </c>
       <c r="M14" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N14" s="12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -1533,16 +1536,16 @@
         <v>345</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L15" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N15" s="12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -1579,16 +1582,16 @@
         <v>100</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L16" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M16" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N16" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -1625,16 +1628,16 @@
         <v>5</v>
       </c>
       <c r="K17" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M17" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N17" s="12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
@@ -1671,16 +1674,16 @@
         <v>180</v>
       </c>
       <c r="K18" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L18" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M18" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N18" s="12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -1717,16 +1720,16 @@
         <v>250</v>
       </c>
       <c r="K19" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L19" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M19" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N19" s="12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -1763,16 +1766,16 @@
         <v>410</v>
       </c>
       <c r="K20" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L20" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M20" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N20" s="12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
@@ -1809,16 +1812,16 @@
         <v>205</v>
       </c>
       <c r="K21" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L21" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="L21" s="11" t="s">
-        <v>62</v>
-      </c>
       <c r="M21" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N21" s="12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
@@ -1855,16 +1858,16 @@
         <v>125</v>
       </c>
       <c r="K22" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L22" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M22" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N22" s="12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -1901,16 +1904,16 @@
         <v>330</v>
       </c>
       <c r="K23" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L23" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M23" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N23" s="12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -1947,16 +1950,16 @@
         <v>340</v>
       </c>
       <c r="K24" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L24" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M24" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N24" s="12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
@@ -1993,16 +1996,16 @@
         <v>471</v>
       </c>
       <c r="K25" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L25" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M25" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N25" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -2039,16 +2042,16 @@
         <v>305</v>
       </c>
       <c r="K26" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="L26" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M26" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N26" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -2085,16 +2088,16 @@
         <v>395</v>
       </c>
       <c r="K27" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L27" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M27" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N27" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -2131,16 +2134,16 @@
         <v>90</v>
       </c>
       <c r="K28" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L28" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M28" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N28" s="12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -2177,16 +2180,16 @@
         <v>325</v>
       </c>
       <c r="K29" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L29" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="M29" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="N29" s="12" t="s">
         <v>85</v>
-      </c>
-      <c r="M29" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="N29" s="12" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -2223,16 +2226,16 @@
         <v>220</v>
       </c>
       <c r="K30" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L30" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M30" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N30" s="12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
@@ -2269,16 +2272,16 @@
         <v>55</v>
       </c>
       <c r="K31" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L31" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M31" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N31" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="32" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -2315,16 +2318,16 @@
         <v>70</v>
       </c>
       <c r="K32" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L32" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M32" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N32" s="12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -2361,16 +2364,16 @@
         <v>270</v>
       </c>
       <c r="K33" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L33" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M33" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N33" s="12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -2407,16 +2410,16 @@
         <v>400</v>
       </c>
       <c r="K34" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L34" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M34" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N34" s="12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -2453,16 +2456,16 @@
         <v>88</v>
       </c>
       <c r="K35" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="L35" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M35" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="L35" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="M35" s="11" t="s">
-        <v>59</v>
-      </c>
       <c r="N35" s="12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -2499,16 +2502,16 @@
         <v>426</v>
       </c>
       <c r="K36" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L36" s="11" t="s">
         <v>60</v>
-      </c>
-      <c r="L36" s="11" t="s">
-        <v>61</v>
       </c>
       <c r="M36" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N36" s="12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="75" x14ac:dyDescent="0.25">
@@ -2545,16 +2548,16 @@
         <v>5</v>
       </c>
       <c r="K37" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L37" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M37" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N37" s="12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="60" x14ac:dyDescent="0.25">
@@ -2591,16 +2594,16 @@
         <v>55</v>
       </c>
       <c r="K38" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L38" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M38" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N38" s="12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -2637,16 +2640,16 @@
         <v>35</v>
       </c>
       <c r="K39" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L39" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M39" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N39" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -2683,16 +2686,16 @@
         <v>185</v>
       </c>
       <c r="K40" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L40" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M40" s="11" t="s">
         <v>49</v>
       </c>
       <c r="N40" s="12" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -2729,39 +2732,63 @@
         <v>515</v>
       </c>
       <c r="K41" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L41" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M41" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="N41" s="12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A42" s="8">
+        <v>46288</v>
+      </c>
+      <c r="B42" s="9">
+        <v>310</v>
+      </c>
+      <c r="C42" s="9">
+        <v>40</v>
+      </c>
+      <c r="D42" s="9">
         <v>60</v>
       </c>
-      <c r="L41" s="11" t="s">
+      <c r="E42" s="9">
+        <v>50</v>
+      </c>
+      <c r="F42" s="9">
+        <v>350</v>
+      </c>
+      <c r="G42" s="9">
+        <v>7</v>
+      </c>
+      <c r="H42" s="9">
+        <v>340</v>
+      </c>
+      <c r="I42" s="10">
+        <f t="shared" si="0"/>
+        <v>1150</v>
+      </c>
+      <c r="J42" s="10">
+        <f t="shared" si="1"/>
+        <v>290</v>
+      </c>
+      <c r="K42" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="L42" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="M41" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="N41" s="12" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A42" s="8"/>
-      <c r="B42" s="9"/>
-      <c r="C42" s="9"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="9"/>
-      <c r="F42" s="9"/>
-      <c r="G42" s="9"/>
-      <c r="H42" s="9"/>
-      <c r="I42" s="10" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J42" s="10" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K42" s="11"/>
-      <c r="L42" s="11"/>
-      <c r="M42" s="11"/>
-      <c r="N42" s="12"/>
+      <c r="M42" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N42" s="12" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="8"/>

</xml_diff>

<commit_message>
Updated Excel - 24 September 2026
</commit_message>
<xml_diff>
--- a/12603165.xlsx
+++ b/12603165.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MINOR PROJECT #1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B5F68E7-742C-4A61-8069-D78C223CA043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B7C9BD4-2DBF-43CD-871A-6ADEDB09F8B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="101">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -332,6 +332,9 @@
   </si>
   <si>
     <t>The day was Too tiring But enjoyed the Lectures.</t>
+  </si>
+  <si>
+    <t>Learned about some deployment tenchiques for Front end projects.</t>
   </si>
 </sst>
 </file>
@@ -2790,27 +2793,51 @@
         <v>99</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A43" s="8"/>
-      <c r="B43" s="9"/>
-      <c r="C43" s="9"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="9"/>
-      <c r="G43" s="9"/>
-      <c r="H43" s="9"/>
-      <c r="I43" s="10" t="str">
+    <row r="43" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A43" s="8">
+        <v>46289</v>
+      </c>
+      <c r="B43" s="9">
+        <v>400</v>
+      </c>
+      <c r="C43" s="9">
+        <v>40</v>
+      </c>
+      <c r="D43" s="9">
+        <v>50</v>
+      </c>
+      <c r="E43" s="9">
+        <v>80</v>
+      </c>
+      <c r="F43" s="9">
+        <v>200</v>
+      </c>
+      <c r="G43" s="9">
+        <v>4</v>
+      </c>
+      <c r="H43" s="9">
+        <v>120</v>
+      </c>
+      <c r="I43" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J43" s="10" t="str">
+        <v>890</v>
+      </c>
+      <c r="J43" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K43" s="11"/>
-      <c r="L43" s="11"/>
-      <c r="M43" s="11"/>
-      <c r="N43" s="12"/>
+        <v>550</v>
+      </c>
+      <c r="K43" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="L43" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="M43" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="N43" s="12" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="8"/>

</xml_diff>

<commit_message>
Updated Excel - 12 September 2026
</commit_message>
<xml_diff>
--- a/12603165.xlsx
+++ b/12603165.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MINOR PROJECT #1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B7C9BD4-2DBF-43CD-871A-6ADEDB09F8B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F61FD5F-1FA4-4C54-A76B-FD92993EFDB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="102">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -335,6 +335,9 @@
   </si>
   <si>
     <t>Learned about some deployment tenchiques for Front end projects.</t>
+  </si>
+  <si>
+    <t>Attended a Meeting with our new clients for website devolopment and media managing.</t>
   </si>
 </sst>
 </file>
@@ -2839,27 +2842,51 @@
         <v>100</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A44" s="8"/>
-      <c r="B44" s="9"/>
-      <c r="C44" s="9"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="9"/>
-      <c r="G44" s="9"/>
-      <c r="H44" s="9"/>
-      <c r="I44" s="10" t="str">
+    <row r="44" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A44" s="8">
+        <v>46290</v>
+      </c>
+      <c r="B44" s="9">
+        <v>300</v>
+      </c>
+      <c r="C44" s="9">
+        <v>45</v>
+      </c>
+      <c r="D44" s="9">
+        <v>110</v>
+      </c>
+      <c r="E44" s="9">
+        <v>50</v>
+      </c>
+      <c r="F44" s="9">
+        <v>300</v>
+      </c>
+      <c r="G44" s="9">
+        <v>6</v>
+      </c>
+      <c r="H44" s="9">
+        <v>300</v>
+      </c>
+      <c r="I44" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J44" s="10" t="str">
+        <v>1105</v>
+      </c>
+      <c r="J44" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K44" s="11"/>
-      <c r="L44" s="11"/>
-      <c r="M44" s="11"/>
-      <c r="N44" s="12"/>
+        <v>335</v>
+      </c>
+      <c r="K44" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="L44" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="M44" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="N44" s="12" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="8"/>

</xml_diff>

<commit_message>
Updated Excel - 26 September 2026
</commit_message>
<xml_diff>
--- a/12603165.xlsx
+++ b/12603165.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MINOR PROJECT #1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F61FD5F-1FA4-4C54-A76B-FD92993EFDB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCA0701-3B76-435B-930E-B19A65265534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="103">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -338,6 +338,9 @@
   </si>
   <si>
     <t>Attended a Meeting with our new clients for website devolopment and media managing.</t>
+  </si>
+  <si>
+    <t>Participated in a 24 hrs Hackathon , and reached 32nd position on evaluation</t>
   </si>
 </sst>
 </file>
@@ -2888,27 +2891,51 @@
         <v>101</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A45" s="8"/>
-      <c r="B45" s="9"/>
-      <c r="C45" s="9"/>
-      <c r="D45" s="9"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="9"/>
-      <c r="G45" s="9"/>
-      <c r="H45" s="9"/>
-      <c r="I45" s="10" t="str">
+    <row r="45" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A45" s="8">
+        <v>46291</v>
+      </c>
+      <c r="B45" s="9">
+        <v>200</v>
+      </c>
+      <c r="C45" s="9">
+        <v>0</v>
+      </c>
+      <c r="D45" s="9">
+        <v>0</v>
+      </c>
+      <c r="E45" s="9">
+        <v>0</v>
+      </c>
+      <c r="F45" s="9">
+        <v>0</v>
+      </c>
+      <c r="G45" s="9">
+        <v>0</v>
+      </c>
+      <c r="H45" s="9">
+        <v>1000</v>
+      </c>
+      <c r="I45" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J45" s="10" t="str">
+        <v>1200</v>
+      </c>
+      <c r="J45" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K45" s="11"/>
-      <c r="L45" s="11"/>
-      <c r="M45" s="11"/>
-      <c r="N45" s="12"/>
+        <v>240</v>
+      </c>
+      <c r="K45" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L45" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M45" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N45" s="12" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="8"/>

</xml_diff>

<commit_message>
Updated Excel - 3 October 2026
</commit_message>
<xml_diff>
--- a/12603165.xlsx
+++ b/12603165.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MINOR PROJECT #1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCA0701-3B76-435B-930E-B19A65265534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7AAF3B8-2C12-478F-8A13-12A53394C9A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="110">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -341,6 +341,27 @@
   </si>
   <si>
     <t>Participated in a 24 hrs Hackathon , and reached 32nd position on evaluation</t>
+  </si>
+  <si>
+    <t>Was very tired after the 24 hrs hackathon so wasn’t able to do much.</t>
+  </si>
+  <si>
+    <t>Situation was not idle in the university so was planning to go home.</t>
+  </si>
+  <si>
+    <t>with no sleep ,WHOLE DAY IN JOURNEY FROM University to home town total 27 Hrs</t>
+  </si>
+  <si>
+    <t>Continued the studies and informations gathering and my designing work simultaneously.</t>
+  </si>
+  <si>
+    <t>Worked on some Ui changes in a Jewellery E commerce Website.</t>
+  </si>
+  <si>
+    <t>Whole day was very productive and amazing</t>
+  </si>
+  <si>
+    <t>Enjoyied the day with my Faimly members.</t>
   </si>
 </sst>
 </file>
@@ -2908,7 +2929,7 @@
         <v>0</v>
       </c>
       <c r="F45" s="9">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="G45" s="9">
         <v>0</v>
@@ -2918,11 +2939,11 @@
       </c>
       <c r="I45" s="10">
         <f t="shared" si="0"/>
-        <v>1200</v>
+        <v>1350</v>
       </c>
       <c r="J45" s="10">
         <f t="shared" si="1"/>
-        <v>240</v>
+        <v>90</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>60</v>
@@ -2937,159 +2958,327 @@
         <v>102</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A46" s="8"/>
-      <c r="B46" s="9"/>
-      <c r="C46" s="9"/>
-      <c r="D46" s="9"/>
-      <c r="E46" s="9"/>
-      <c r="F46" s="9"/>
-      <c r="G46" s="9"/>
-      <c r="H46" s="9"/>
-      <c r="I46" s="10" t="str">
+    <row r="46" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A46" s="8">
+        <v>46292</v>
+      </c>
+      <c r="B46" s="9">
+        <v>150</v>
+      </c>
+      <c r="C46" s="9">
+        <v>45</v>
+      </c>
+      <c r="D46" s="9">
+        <v>0</v>
+      </c>
+      <c r="E46" s="9">
+        <v>0</v>
+      </c>
+      <c r="F46" s="9">
+        <v>0</v>
+      </c>
+      <c r="G46" s="9">
+        <v>0</v>
+      </c>
+      <c r="H46" s="9">
+        <v>900</v>
+      </c>
+      <c r="I46" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J46" s="10" t="str">
+        <v>1095</v>
+      </c>
+      <c r="J46" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K46" s="11"/>
-      <c r="L46" s="11"/>
-      <c r="M46" s="11"/>
-      <c r="N46" s="12"/>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A47" s="8"/>
-      <c r="B47" s="9"/>
-      <c r="C47" s="9"/>
-      <c r="D47" s="9"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="9"/>
-      <c r="G47" s="9"/>
-      <c r="H47" s="9"/>
-      <c r="I47" s="10" t="str">
+        <v>345</v>
+      </c>
+      <c r="K46" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="L46" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="M46" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="N46" s="12" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A47" s="8">
+        <v>46293</v>
+      </c>
+      <c r="B47" s="9">
+        <v>0</v>
+      </c>
+      <c r="C47" s="9">
+        <v>0</v>
+      </c>
+      <c r="D47" s="9">
+        <v>0</v>
+      </c>
+      <c r="E47" s="9">
+        <v>0</v>
+      </c>
+      <c r="F47" s="9">
+        <v>0</v>
+      </c>
+      <c r="G47" s="9">
+        <v>0</v>
+      </c>
+      <c r="H47" s="9">
+        <v>1300</v>
+      </c>
+      <c r="I47" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J47" s="10" t="str">
+        <v>1300</v>
+      </c>
+      <c r="J47" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K47" s="11"/>
-      <c r="L47" s="11"/>
-      <c r="M47" s="11"/>
-      <c r="N47" s="12"/>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A48" s="8"/>
-      <c r="B48" s="9"/>
-      <c r="C48" s="9"/>
-      <c r="D48" s="9"/>
-      <c r="E48" s="9"/>
-      <c r="F48" s="9"/>
-      <c r="G48" s="9"/>
-      <c r="H48" s="9"/>
-      <c r="I48" s="10" t="str">
+        <v>140</v>
+      </c>
+      <c r="K47" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="L47" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="M47" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N47" s="12" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A48" s="8">
+        <v>46294</v>
+      </c>
+      <c r="B48" s="9">
+        <v>300</v>
+      </c>
+      <c r="C48" s="9">
+        <v>40</v>
+      </c>
+      <c r="D48" s="9">
+        <v>90</v>
+      </c>
+      <c r="E48" s="9">
+        <v>60</v>
+      </c>
+      <c r="F48" s="9">
+        <v>0</v>
+      </c>
+      <c r="G48" s="9">
+        <v>0</v>
+      </c>
+      <c r="H48" s="9">
+        <v>300</v>
+      </c>
+      <c r="I48" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J48" s="10" t="str">
+        <v>790</v>
+      </c>
+      <c r="J48" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K48" s="11"/>
-      <c r="L48" s="11"/>
-      <c r="M48" s="11"/>
-      <c r="N48" s="12"/>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A49" s="8"/>
-      <c r="B49" s="9"/>
-      <c r="C49" s="9"/>
-      <c r="D49" s="9"/>
-      <c r="E49" s="9"/>
-      <c r="F49" s="9"/>
-      <c r="G49" s="9"/>
-      <c r="H49" s="9"/>
-      <c r="I49" s="10" t="str">
+        <v>650</v>
+      </c>
+      <c r="K48" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="L48" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="M48" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="N48" s="12" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A49" s="8">
+        <v>46295</v>
+      </c>
+      <c r="B49" s="9">
+        <v>450</v>
+      </c>
+      <c r="C49" s="9">
+        <v>40</v>
+      </c>
+      <c r="D49" s="9">
+        <v>120</v>
+      </c>
+      <c r="E49" s="9">
+        <v>80</v>
+      </c>
+      <c r="F49" s="9">
+        <v>0</v>
+      </c>
+      <c r="G49" s="9">
+        <v>0</v>
+      </c>
+      <c r="H49" s="9">
+        <v>450</v>
+      </c>
+      <c r="I49" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J49" s="10" t="str">
+        <v>1140</v>
+      </c>
+      <c r="J49" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K49" s="11"/>
-      <c r="L49" s="11"/>
-      <c r="M49" s="11"/>
-      <c r="N49" s="12"/>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A50" s="8"/>
-      <c r="B50" s="9"/>
-      <c r="C50" s="9"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="9"/>
-      <c r="F50" s="9"/>
-      <c r="G50" s="9"/>
-      <c r="H50" s="9"/>
-      <c r="I50" s="10" t="str">
+        <v>300</v>
+      </c>
+      <c r="K49" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="L49" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M49" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N49" s="12" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A50" s="8">
+        <v>46296</v>
+      </c>
+      <c r="B50" s="9">
+        <v>300</v>
+      </c>
+      <c r="C50" s="9">
+        <v>45</v>
+      </c>
+      <c r="D50" s="9">
+        <v>130</v>
+      </c>
+      <c r="E50" s="9">
+        <v>65</v>
+      </c>
+      <c r="F50" s="9">
+        <v>0</v>
+      </c>
+      <c r="G50" s="9">
+        <v>0</v>
+      </c>
+      <c r="H50" s="9">
+        <v>300</v>
+      </c>
+      <c r="I50" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J50" s="10" t="str">
+        <v>840</v>
+      </c>
+      <c r="J50" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K50" s="11"/>
-      <c r="L50" s="11"/>
-      <c r="M50" s="11"/>
-      <c r="N50" s="12"/>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A51" s="8"/>
-      <c r="B51" s="9"/>
-      <c r="C51" s="9"/>
-      <c r="D51" s="9"/>
-      <c r="E51" s="9"/>
-      <c r="F51" s="9"/>
-      <c r="G51" s="9"/>
-      <c r="H51" s="9"/>
-      <c r="I51" s="10" t="str">
+        <v>600</v>
+      </c>
+      <c r="K50" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L50" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="M50" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="N50" s="12" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A51" s="8">
+        <v>46297</v>
+      </c>
+      <c r="B51" s="9">
+        <v>360</v>
+      </c>
+      <c r="C51" s="9">
+        <v>40</v>
+      </c>
+      <c r="D51" s="9">
+        <v>150</v>
+      </c>
+      <c r="E51" s="9">
+        <v>95</v>
+      </c>
+      <c r="F51" s="9">
+        <v>0</v>
+      </c>
+      <c r="G51" s="9">
+        <v>0</v>
+      </c>
+      <c r="H51" s="9">
+        <v>510</v>
+      </c>
+      <c r="I51" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J51" s="10" t="str">
+        <v>1155</v>
+      </c>
+      <c r="J51" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K51" s="11"/>
-      <c r="L51" s="11"/>
-      <c r="M51" s="11"/>
-      <c r="N51" s="12"/>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A52" s="8"/>
-      <c r="B52" s="9"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="9"/>
-      <c r="F52" s="9"/>
-      <c r="G52" s="9"/>
-      <c r="H52" s="9"/>
-      <c r="I52" s="10" t="str">
+        <v>285</v>
+      </c>
+      <c r="K51" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L51" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M51" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="N51" s="12" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A52" s="8">
+        <v>46298</v>
+      </c>
+      <c r="B52" s="9">
+        <v>390</v>
+      </c>
+      <c r="C52" s="9">
+        <v>45</v>
+      </c>
+      <c r="D52" s="9">
+        <v>120</v>
+      </c>
+      <c r="E52" s="9">
+        <v>110</v>
+      </c>
+      <c r="F52" s="9">
+        <v>0</v>
+      </c>
+      <c r="G52" s="9">
+        <v>0</v>
+      </c>
+      <c r="H52" s="9">
+        <v>560</v>
+      </c>
+      <c r="I52" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J52" s="10" t="str">
+        <v>1225</v>
+      </c>
+      <c r="J52" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K52" s="11"/>
-      <c r="L52" s="11"/>
-      <c r="M52" s="11"/>
-      <c r="N52" s="12"/>
+        <v>215</v>
+      </c>
+      <c r="K52" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="L52" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="M52" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="N52" s="12" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="8"/>

</xml_diff>

<commit_message>
Updated excel - 5 September 2026
</commit_message>
<xml_diff>
--- a/12603165.xlsx
+++ b/12603165.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\12603165-CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB58EE24-0598-4B8B-B669-87ABB18030DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AA6E2E7-7D24-4195-B16C-E3725C7EC9B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="112">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -365,6 +365,9 @@
   </si>
   <si>
     <t>Started Preparing for my Mid term examinations.</t>
+  </si>
+  <si>
+    <t>tried some new routing techniques on cisco packet tracer.</t>
   </si>
 </sst>
 </file>
@@ -3329,27 +3332,51 @@
         <v>110</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A54" s="8"/>
-      <c r="B54" s="9"/>
-      <c r="C54" s="9"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="9"/>
-      <c r="F54" s="9"/>
-      <c r="G54" s="9"/>
-      <c r="H54" s="9"/>
-      <c r="I54" s="10" t="str">
+    <row r="54" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A54" s="8">
+        <v>46300</v>
+      </c>
+      <c r="B54" s="9">
+        <v>300</v>
+      </c>
+      <c r="C54" s="9">
+        <v>55</v>
+      </c>
+      <c r="D54" s="9">
+        <v>220</v>
+      </c>
+      <c r="E54" s="9">
+        <v>90</v>
+      </c>
+      <c r="F54" s="9">
+        <v>0</v>
+      </c>
+      <c r="G54" s="9">
+        <v>0</v>
+      </c>
+      <c r="H54" s="9">
+        <v>300</v>
+      </c>
+      <c r="I54" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J54" s="10" t="str">
+        <v>965</v>
+      </c>
+      <c r="J54" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K54" s="11"/>
-      <c r="L54" s="11"/>
-      <c r="M54" s="11"/>
-      <c r="N54" s="12"/>
+        <v>475</v>
+      </c>
+      <c r="K54" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L54" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M54" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N54" s="12" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="8"/>

</xml_diff>

<commit_message>
Updated Excel - 6 September
</commit_message>
<xml_diff>
--- a/12603165.xlsx
+++ b/12603165.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\12603165-CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AA6E2E7-7D24-4195-B16C-E3725C7EC9B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{639F0726-75A3-4693-AA0A-92E8182BFC80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="113">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -368,6 +368,9 @@
   </si>
   <si>
     <t>tried some new routing techniques on cisco packet tracer.</t>
+  </si>
+  <si>
+    <t>Reviewed my daily progress and noticed the areas that need more practice during the holidays.</t>
   </si>
 </sst>
 </file>
@@ -3378,27 +3381,51 @@
         <v>111</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A55" s="8"/>
-      <c r="B55" s="9"/>
-      <c r="C55" s="9"/>
-      <c r="D55" s="9"/>
-      <c r="E55" s="9"/>
-      <c r="F55" s="9"/>
-      <c r="G55" s="9"/>
-      <c r="H55" s="9"/>
-      <c r="I55" s="10" t="str">
+    <row r="55" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A55" s="8">
+        <v>46301</v>
+      </c>
+      <c r="B55" s="9">
+        <v>340</v>
+      </c>
+      <c r="C55" s="9">
+        <v>50</v>
+      </c>
+      <c r="D55" s="9">
+        <v>160</v>
+      </c>
+      <c r="E55" s="9">
+        <v>130</v>
+      </c>
+      <c r="F55" s="9">
+        <v>0</v>
+      </c>
+      <c r="G55" s="9">
+        <v>0</v>
+      </c>
+      <c r="H55" s="9">
+        <v>460</v>
+      </c>
+      <c r="I55" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J55" s="10" t="str">
+        <v>1140</v>
+      </c>
+      <c r="J55" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K55" s="11"/>
-      <c r="L55" s="11"/>
-      <c r="M55" s="11"/>
-      <c r="N55" s="12"/>
+        <v>300</v>
+      </c>
+      <c r="K55" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L55" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M55" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="N55" s="12" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="8"/>

</xml_diff>

<commit_message>
Updated Excel 8 september
</commit_message>
<xml_diff>
--- a/12603165.xlsx
+++ b/12603165.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\12603165-CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{639F0726-75A3-4693-AA0A-92E8182BFC80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A07EAC9-8F92-4BDE-88F8-A9C17924E78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="115">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -371,6 +371,12 @@
   </si>
   <si>
     <t>Reviewed my daily progress and noticed the areas that need more practice during the holidays.</t>
+  </si>
+  <si>
+    <t>Had some discussions for new marketing techniques for A hospital.</t>
+  </si>
+  <si>
+    <t>Started revision for the topics taught in online classes for Exams.</t>
   </si>
 </sst>
 </file>
@@ -3352,21 +3358,21 @@
         <v>90</v>
       </c>
       <c r="F54" s="9">
-        <v>0</v>
+        <v>350</v>
       </c>
       <c r="G54" s="9">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H54" s="9">
         <v>300</v>
       </c>
       <c r="I54" s="10">
         <f t="shared" si="0"/>
-        <v>965</v>
+        <v>1315</v>
       </c>
       <c r="J54" s="10">
         <f t="shared" si="1"/>
-        <v>475</v>
+        <v>125</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>59</v>
@@ -3398,21 +3404,21 @@
         <v>130</v>
       </c>
       <c r="F55" s="9">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="G55" s="9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H55" s="9">
         <v>460</v>
       </c>
       <c r="I55" s="10">
         <f t="shared" si="0"/>
-        <v>1140</v>
+        <v>1290</v>
       </c>
       <c r="J55" s="10">
         <f t="shared" si="1"/>
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>59</v>
@@ -3427,49 +3433,97 @@
         <v>112</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A56" s="8"/>
-      <c r="B56" s="9"/>
-      <c r="C56" s="9"/>
-      <c r="D56" s="9"/>
-      <c r="E56" s="9"/>
-      <c r="F56" s="9"/>
-      <c r="G56" s="9"/>
-      <c r="H56" s="9"/>
-      <c r="I56" s="10" t="str">
+    <row r="56" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A56" s="8">
+        <v>46302</v>
+      </c>
+      <c r="B56" s="9">
+        <v>420</v>
+      </c>
+      <c r="C56" s="9">
+        <v>45</v>
+      </c>
+      <c r="D56" s="9">
+        <v>150</v>
+      </c>
+      <c r="E56" s="9">
+        <v>80</v>
+      </c>
+      <c r="F56" s="9">
+        <v>350</v>
+      </c>
+      <c r="G56" s="9">
+        <v>7</v>
+      </c>
+      <c r="H56" s="9">
+        <v>300</v>
+      </c>
+      <c r="I56" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J56" s="10" t="str">
+        <v>1345</v>
+      </c>
+      <c r="J56" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K56" s="11"/>
-      <c r="L56" s="11"/>
-      <c r="M56" s="11"/>
-      <c r="N56" s="12"/>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A57" s="8"/>
-      <c r="B57" s="9"/>
-      <c r="C57" s="9"/>
-      <c r="D57" s="9"/>
-      <c r="E57" s="9"/>
-      <c r="F57" s="9"/>
-      <c r="G57" s="9"/>
-      <c r="H57" s="9"/>
-      <c r="I57" s="10" t="str">
+        <v>95</v>
+      </c>
+      <c r="K56" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L56" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="M56" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="N56" s="12" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A57" s="8">
+        <v>46303</v>
+      </c>
+      <c r="B57" s="9">
+        <v>410</v>
+      </c>
+      <c r="C57" s="9">
+        <v>55</v>
+      </c>
+      <c r="D57" s="9">
+        <v>160</v>
+      </c>
+      <c r="E57" s="9">
+        <v>50</v>
+      </c>
+      <c r="F57" s="9">
+        <v>0</v>
+      </c>
+      <c r="G57" s="9">
+        <v>0</v>
+      </c>
+      <c r="H57" s="9">
+        <v>450</v>
+      </c>
+      <c r="I57" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J57" s="10" t="str">
+        <v>1125</v>
+      </c>
+      <c r="J57" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K57" s="11"/>
-      <c r="L57" s="11"/>
-      <c r="M57" s="11"/>
-      <c r="N57" s="12"/>
+        <v>315</v>
+      </c>
+      <c r="K57" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="L57" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="M57" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N57" s="12" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" s="8"/>

</xml_diff>

<commit_message>
Updated Excel 15th September
</commit_message>
<xml_diff>
--- a/12603165.xlsx
+++ b/12603165.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\12603165-CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A07EAC9-8F92-4BDE-88F8-A9C17924E78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6591E74E-26B4-4D22-97F7-A5E332775C66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="122">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -377,6 +377,27 @@
   </si>
   <si>
     <t>Started revision for the topics taught in online classes for Exams.</t>
+  </si>
+  <si>
+    <t>had to travel back to University , That took too 26 hrs .</t>
+  </si>
+  <si>
+    <t>Was really tired because almost no sleep in night and travell fatigue.</t>
+  </si>
+  <si>
+    <t>Worked On some existing codes for more readibility.</t>
+  </si>
+  <si>
+    <t>The Networking Exam  went well then expected.</t>
+  </si>
+  <si>
+    <t>The C++ exam was fine a bit Moderate level , So I made up my mind to give extra focus on The course.</t>
+  </si>
+  <si>
+    <t>Gave the Database Exam covienently and gained good confidence in the subject.</t>
+  </si>
+  <si>
+    <t>Solved Almost All question of 1st an 2nd level IN aptitude to get good command.</t>
   </si>
 </sst>
 </file>
@@ -3525,159 +3546,327 @@
         <v>114</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A58" s="8"/>
-      <c r="B58" s="9"/>
-      <c r="C58" s="9"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="9"/>
-      <c r="F58" s="9"/>
-      <c r="G58" s="9"/>
-      <c r="H58" s="9"/>
-      <c r="I58" s="10" t="str">
+    <row r="58" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A58" s="8">
+        <v>46304</v>
+      </c>
+      <c r="B58" s="9">
+        <v>270</v>
+      </c>
+      <c r="C58" s="9">
+        <v>0</v>
+      </c>
+      <c r="D58" s="9">
+        <v>0</v>
+      </c>
+      <c r="E58" s="9">
+        <v>0</v>
+      </c>
+      <c r="F58" s="9">
+        <v>0</v>
+      </c>
+      <c r="G58" s="9">
+        <v>0</v>
+      </c>
+      <c r="H58" s="9">
+        <v>1000</v>
+      </c>
+      <c r="I58" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J58" s="10" t="str">
+        <v>1270</v>
+      </c>
+      <c r="J58" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K58" s="11"/>
-      <c r="L58" s="11"/>
-      <c r="M58" s="11"/>
-      <c r="N58" s="12"/>
-    </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A59" s="8"/>
-      <c r="B59" s="9"/>
-      <c r="C59" s="9"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="9"/>
-      <c r="G59" s="9"/>
-      <c r="H59" s="9"/>
-      <c r="I59" s="10" t="str">
+        <v>170</v>
+      </c>
+      <c r="K58" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L58" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="M58" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N58" s="12" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A59" s="8">
+        <v>46305</v>
+      </c>
+      <c r="B59" s="9">
+        <v>240</v>
+      </c>
+      <c r="C59" s="9">
+        <v>0</v>
+      </c>
+      <c r="D59" s="9">
+        <v>40</v>
+      </c>
+      <c r="E59" s="9">
+        <v>50</v>
+      </c>
+      <c r="F59" s="9">
+        <v>0</v>
+      </c>
+      <c r="G59" s="9">
+        <v>0</v>
+      </c>
+      <c r="H59" s="9">
+        <v>500</v>
+      </c>
+      <c r="I59" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J59" s="10" t="str">
+        <v>830</v>
+      </c>
+      <c r="J59" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K59" s="11"/>
-      <c r="L59" s="11"/>
-      <c r="M59" s="11"/>
-      <c r="N59" s="12"/>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A60" s="8"/>
-      <c r="B60" s="9"/>
-      <c r="C60" s="9"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="9"/>
-      <c r="F60" s="9"/>
-      <c r="G60" s="9"/>
-      <c r="H60" s="9"/>
-      <c r="I60" s="10" t="str">
+        <v>610</v>
+      </c>
+      <c r="K59" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L59" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="M59" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="N59" s="12" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A60" s="8">
+        <v>46306</v>
+      </c>
+      <c r="B60" s="9">
+        <v>320</v>
+      </c>
+      <c r="C60" s="9">
+        <v>45</v>
+      </c>
+      <c r="D60" s="9">
+        <v>360</v>
+      </c>
+      <c r="E60" s="9">
+        <v>150</v>
+      </c>
+      <c r="F60" s="9">
+        <v>0</v>
+      </c>
+      <c r="G60" s="9">
+        <v>0</v>
+      </c>
+      <c r="H60" s="9">
+        <v>200</v>
+      </c>
+      <c r="I60" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J60" s="10" t="str">
+        <v>1075</v>
+      </c>
+      <c r="J60" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K60" s="11"/>
-      <c r="L60" s="11"/>
-      <c r="M60" s="11"/>
-      <c r="N60" s="12"/>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A61" s="8"/>
-      <c r="B61" s="9"/>
-      <c r="C61" s="9"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="9"/>
-      <c r="F61" s="9"/>
-      <c r="G61" s="9"/>
-      <c r="H61" s="9"/>
-      <c r="I61" s="10" t="str">
+        <v>365</v>
+      </c>
+      <c r="K60" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="L60" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M60" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N60" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A61" s="8">
+        <v>46307</v>
+      </c>
+      <c r="B61" s="9">
+        <v>360</v>
+      </c>
+      <c r="C61" s="9">
+        <v>40</v>
+      </c>
+      <c r="D61" s="9">
+        <v>390</v>
+      </c>
+      <c r="E61" s="9">
+        <v>60</v>
+      </c>
+      <c r="F61" s="9">
+        <v>0</v>
+      </c>
+      <c r="G61" s="9">
+        <v>0</v>
+      </c>
+      <c r="H61" s="9">
+        <v>200</v>
+      </c>
+      <c r="I61" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J61" s="10" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J61" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K61" s="11"/>
-      <c r="L61" s="11"/>
-      <c r="M61" s="11"/>
-      <c r="N61" s="12"/>
-    </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A62" s="8"/>
-      <c r="B62" s="9"/>
-      <c r="C62" s="9"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="9"/>
-      <c r="F62" s="9"/>
-      <c r="G62" s="9"/>
-      <c r="H62" s="9"/>
-      <c r="I62" s="10" t="str">
+        <v>390</v>
+      </c>
+      <c r="K61" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="L61" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="M61" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N61" s="12" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A62" s="8">
+        <v>46308</v>
+      </c>
+      <c r="B62" s="9">
+        <v>300</v>
+      </c>
+      <c r="C62" s="9">
+        <v>40</v>
+      </c>
+      <c r="D62" s="9">
+        <v>300</v>
+      </c>
+      <c r="E62" s="9">
+        <v>140</v>
+      </c>
+      <c r="F62" s="9">
+        <v>0</v>
+      </c>
+      <c r="G62" s="9">
+        <v>0</v>
+      </c>
+      <c r="H62" s="9">
+        <v>260</v>
+      </c>
+      <c r="I62" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J62" s="10" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J62" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K62" s="11"/>
-      <c r="L62" s="11"/>
-      <c r="M62" s="11"/>
-      <c r="N62" s="12"/>
-    </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A63" s="8"/>
-      <c r="B63" s="9"/>
-      <c r="C63" s="9"/>
-      <c r="D63" s="9"/>
-      <c r="E63" s="9"/>
-      <c r="F63" s="9"/>
-      <c r="G63" s="9"/>
-      <c r="H63" s="9"/>
-      <c r="I63" s="10" t="str">
+        <v>400</v>
+      </c>
+      <c r="K62" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="L62" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M62" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="N62" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A63" s="8">
+        <v>46309</v>
+      </c>
+      <c r="B63" s="9">
+        <v>300</v>
+      </c>
+      <c r="C63" s="9">
+        <v>45</v>
+      </c>
+      <c r="D63" s="9">
+        <v>410</v>
+      </c>
+      <c r="E63" s="9">
+        <v>50</v>
+      </c>
+      <c r="F63" s="9">
+        <v>0</v>
+      </c>
+      <c r="G63" s="9">
+        <v>0</v>
+      </c>
+      <c r="H63" s="9">
+        <v>210</v>
+      </c>
+      <c r="I63" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J63" s="10" t="str">
+        <v>1015</v>
+      </c>
+      <c r="J63" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K63" s="11"/>
-      <c r="L63" s="11"/>
-      <c r="M63" s="11"/>
-      <c r="N63" s="12"/>
-    </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A64" s="8"/>
-      <c r="B64" s="9"/>
-      <c r="C64" s="9"/>
-      <c r="D64" s="9"/>
-      <c r="E64" s="9"/>
-      <c r="F64" s="9"/>
-      <c r="G64" s="9"/>
-      <c r="H64" s="9"/>
-      <c r="I64" s="10" t="str">
+        <v>425</v>
+      </c>
+      <c r="K63" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="L63" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M63" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N63" s="12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A64" s="8">
+        <v>46310</v>
+      </c>
+      <c r="B64" s="9">
+        <v>300</v>
+      </c>
+      <c r="C64" s="9">
+        <v>45</v>
+      </c>
+      <c r="D64" s="9">
+        <v>600</v>
+      </c>
+      <c r="E64" s="9">
+        <v>30</v>
+      </c>
+      <c r="F64" s="9">
+        <v>0</v>
+      </c>
+      <c r="G64" s="9">
+        <v>0</v>
+      </c>
+      <c r="H64" s="9">
+        <v>160</v>
+      </c>
+      <c r="I64" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J64" s="10" t="str">
+        <v>1135</v>
+      </c>
+      <c r="J64" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K64" s="11"/>
-      <c r="L64" s="11"/>
-      <c r="M64" s="11"/>
-      <c r="N64" s="12"/>
+        <v>305</v>
+      </c>
+      <c r="K64" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L64" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M64" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N64" s="12" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="8"/>
@@ -11058,4 +11247,205 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F0F845B241C40547964E628A3A9FD4D5" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="26ddc77cb2d0308c67bc97ebe2bcdb81">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="263ac7fe-287e-4d66-a581-4ec0c8da0161" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c61004864e1595b4a8427a69c7f15600" ns3:_="">
+    <xsd:import namespace="263ac7fe-287e-4d66-a581-4ec0c8da0161"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns3:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSearchProperties" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="263ac7fe-287e-4d66-a581-4ec0c8da0161" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceDateTaken" ma:index="8" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="10" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="11" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE21CED1-6B9A-4824-8B9E-43D7E21FEEB3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="263ac7fe-287e-4d66-a581-4ec0c8da0161"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45EF36EA-A553-4F9D-BCFB-2108914EAC0E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D6656C2-1A4B-4D7E-882E-8F2A959DC7AD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="263ac7fe-287e-4d66-a581-4ec0c8da0161"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated Excel 20th September
</commit_message>
<xml_diff>
--- a/12603165.xlsx
+++ b/12603165.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\12603165-CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6591E74E-26B4-4D22-97F7-A5E332775C66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF67CB48-4CCA-4CED-A2C5-0005E4089B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
     <sheet name="Daily Log" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="127">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -398,6 +398,21 @@
   </si>
   <si>
     <t>Solved Almost All question of 1st an 2nd level IN aptitude to get good command.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">was Skeptical about how my Analytical exam went. </t>
+  </si>
+  <si>
+    <t>Todays English exam went very well and was happy about The Midterms being Over.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Started a New Way of Utilising my time after the midterms to Compete and complete in my own Goals. </t>
+  </si>
+  <si>
+    <t>The day was tiring and was very much demotivaed , but Got back to my usual stuff.</t>
+  </si>
+  <si>
+    <t>As for Previous day Demotivation ,I decided to Experience something new so went out with some of my friends , to get fresh air and do some fun things to get beck to being fully motivated towards our goals.</t>
   </si>
 </sst>
 </file>
@@ -3868,115 +3883,235 @@
         <v>121</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A65" s="8"/>
-      <c r="B65" s="9"/>
-      <c r="C65" s="9"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="9"/>
-      <c r="F65" s="9"/>
-      <c r="G65" s="9"/>
-      <c r="H65" s="9"/>
-      <c r="I65" s="10" t="str">
+    <row r="65" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A65" s="8">
+        <v>46311</v>
+      </c>
+      <c r="B65" s="9">
+        <v>320</v>
+      </c>
+      <c r="C65" s="9">
+        <v>40</v>
+      </c>
+      <c r="D65" s="9">
+        <v>590</v>
+      </c>
+      <c r="E65" s="9">
+        <v>30</v>
+      </c>
+      <c r="F65" s="9">
+        <v>0</v>
+      </c>
+      <c r="G65" s="9">
+        <v>0</v>
+      </c>
+      <c r="H65" s="9">
+        <v>90</v>
+      </c>
+      <c r="I65" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J65" s="10" t="str">
+        <v>1070</v>
+      </c>
+      <c r="J65" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K65" s="11"/>
-      <c r="L65" s="11"/>
-      <c r="M65" s="11"/>
-      <c r="N65" s="12"/>
-    </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A66" s="8"/>
-      <c r="B66" s="9"/>
-      <c r="C66" s="9"/>
-      <c r="D66" s="9"/>
-      <c r="E66" s="9"/>
-      <c r="F66" s="9"/>
-      <c r="G66" s="9"/>
-      <c r="H66" s="9"/>
-      <c r="I66" s="10" t="str">
+        <v>370</v>
+      </c>
+      <c r="K65" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="L65" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M65" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N65" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A66" s="8">
+        <v>46312</v>
+      </c>
+      <c r="B66" s="9">
+        <v>330</v>
+      </c>
+      <c r="C66" s="9">
+        <v>45</v>
+      </c>
+      <c r="D66" s="9">
+        <v>620</v>
+      </c>
+      <c r="E66" s="9">
+        <v>40</v>
+      </c>
+      <c r="F66" s="9">
+        <v>0</v>
+      </c>
+      <c r="G66" s="9">
+        <v>0</v>
+      </c>
+      <c r="H66" s="9">
+        <v>120</v>
+      </c>
+      <c r="I66" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J66" s="10" t="str">
+        <v>1155</v>
+      </c>
+      <c r="J66" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K66" s="11"/>
-      <c r="L66" s="11"/>
-      <c r="M66" s="11"/>
-      <c r="N66" s="12"/>
-    </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A67" s="8"/>
-      <c r="B67" s="9"/>
-      <c r="C67" s="9"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="9"/>
-      <c r="F67" s="9"/>
-      <c r="G67" s="9"/>
-      <c r="H67" s="9"/>
-      <c r="I67" s="10" t="str">
+        <v>285</v>
+      </c>
+      <c r="K66" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L66" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="M66" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N66" s="12" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A67" s="8">
+        <v>46313</v>
+      </c>
+      <c r="B67" s="9">
+        <v>310</v>
+      </c>
+      <c r="C67" s="9">
+        <v>45</v>
+      </c>
+      <c r="D67" s="9">
+        <v>450</v>
+      </c>
+      <c r="E67" s="9">
+        <v>190</v>
+      </c>
+      <c r="F67" s="9">
+        <v>0</v>
+      </c>
+      <c r="G67" s="9">
+        <v>0</v>
+      </c>
+      <c r="H67" s="9">
+        <v>240</v>
+      </c>
+      <c r="I67" s="10">
         <f t="shared" ref="I67:I130" si="2">IF(SUM(B67:F67,H67)=0,"",SUM(B67:F67,H67))</f>
-        <v/>
-      </c>
-      <c r="J67" s="10" t="str">
+        <v>1235</v>
+      </c>
+      <c r="J67" s="10">
         <f t="shared" ref="J67:J130" si="3">IF(I67="","",1440-I67)</f>
-        <v/>
-      </c>
-      <c r="K67" s="11"/>
-      <c r="L67" s="11"/>
-      <c r="M67" s="11"/>
-      <c r="N67" s="12"/>
-    </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A68" s="8"/>
-      <c r="B68" s="9"/>
-      <c r="C68" s="9"/>
-      <c r="D68" s="9"/>
-      <c r="E68" s="9"/>
-      <c r="F68" s="9"/>
-      <c r="G68" s="9"/>
-      <c r="H68" s="9"/>
-      <c r="I68" s="10" t="str">
+        <v>205</v>
+      </c>
+      <c r="K67" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L67" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="M67" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N67" s="12" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A68" s="8">
+        <v>46314</v>
+      </c>
+      <c r="B68" s="9">
+        <v>340</v>
+      </c>
+      <c r="C68" s="9">
+        <v>40</v>
+      </c>
+      <c r="D68" s="9">
+        <v>220</v>
+      </c>
+      <c r="E68" s="9">
+        <v>130</v>
+      </c>
+      <c r="F68" s="9">
+        <v>350</v>
+      </c>
+      <c r="G68" s="9">
+        <v>7</v>
+      </c>
+      <c r="H68" s="9">
+        <v>130</v>
+      </c>
+      <c r="I68" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J68" s="10" t="str">
+        <v>1210</v>
+      </c>
+      <c r="J68" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K68" s="11"/>
-      <c r="L68" s="11"/>
-      <c r="M68" s="11"/>
-      <c r="N68" s="12"/>
-    </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A69" s="8"/>
-      <c r="B69" s="9"/>
-      <c r="C69" s="9"/>
-      <c r="D69" s="9"/>
-      <c r="E69" s="9"/>
-      <c r="F69" s="9"/>
-      <c r="G69" s="9"/>
-      <c r="H69" s="9"/>
-      <c r="I69" s="10" t="str">
+        <v>230</v>
+      </c>
+      <c r="K68" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="L68" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="M68" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="N68" s="12" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+      <c r="A69" s="8">
+        <v>46315</v>
+      </c>
+      <c r="B69" s="9">
+        <v>290</v>
+      </c>
+      <c r="C69" s="9">
+        <v>45</v>
+      </c>
+      <c r="D69" s="9">
+        <v>410</v>
+      </c>
+      <c r="E69" s="9">
+        <v>140</v>
+      </c>
+      <c r="F69" s="9">
+        <v>0</v>
+      </c>
+      <c r="G69" s="9">
+        <v>0</v>
+      </c>
+      <c r="H69" s="9">
+        <v>500</v>
+      </c>
+      <c r="I69" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J69" s="10" t="str">
+        <v>1385</v>
+      </c>
+      <c r="J69" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K69" s="11"/>
-      <c r="L69" s="11"/>
-      <c r="M69" s="11"/>
-      <c r="N69" s="12"/>
+        <v>55</v>
+      </c>
+      <c r="K69" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L69" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="M69" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="N69" s="12" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" s="8"/>
@@ -11250,6 +11385,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F0F845B241C40547964E628A3A9FD4D5" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="26ddc77cb2d0308c67bc97ebe2bcdb81">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="263ac7fe-287e-4d66-a581-4ec0c8da0161" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c61004864e1595b4a8427a69c7f15600" ns3:_="">
     <xsd:import namespace="263ac7fe-287e-4d66-a581-4ec0c8da0161"/>
@@ -11393,22 +11543,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D6656C2-1A4B-4D7E-882E-8F2A959DC7AD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="263ac7fe-287e-4d66-a581-4ec0c8da0161"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45EF36EA-A553-4F9D-BCFB-2108914EAC0E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE21CED1-6B9A-4824-8B9E-43D7E21FEEB3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11424,28 +11583,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45EF36EA-A553-4F9D-BCFB-2108914EAC0E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D6656C2-1A4B-4D7E-882E-8F2A959DC7AD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="263ac7fe-287e-4d66-a581-4ec0c8da0161"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>